<commit_message>
Update data_import_example spreadsheet with small fixes.
</commit_message>
<xml_diff>
--- a/docs/data_import_example.xlsx
+++ b/docs/data_import_example.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="28"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="34"/>
   </bookViews>
   <sheets>
     <sheet name="Locations" sheetId="1" state="visible" r:id="rId2"/>
@@ -42,7 +42,7 @@
     <sheet name="Critical Illness Plans" sheetId="32" state="visible" r:id="rId33"/>
     <sheet name="Cancer Plans" sheetId="33" state="visible" r:id="rId34"/>
     <sheet name="Accident Plans" sheetId="34" state="visible" r:id="rId35"/>
-    <sheet name="Hospital Confiement Plans" sheetId="35" state="visible" r:id="rId36"/>
+    <sheet name="Hospital Confinement Plans" sheetId="35" state="visible" r:id="rId36"/>
     <sheet name="Parking and Transit Plans" sheetId="36" state="visible" r:id="rId37"/>
     <sheet name="Identity Theft Plans" sheetId="37" state="visible" r:id="rId38"/>
     <sheet name="Enrollments" sheetId="38" state="visible" r:id="rId39"/>
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="927" uniqueCount="322">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="935" uniqueCount="323">
   <si>
     <t xml:space="preserve">code</t>
   </si>
@@ -752,6 +752,9 @@
   </si>
   <si>
     <t xml:space="preserve">employee assistance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">http://eap.com</t>
   </si>
   <si>
     <t xml:space="preserve">LTC234</t>
@@ -5017,7 +5020,8 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="15.94"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="6.73"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="0" width="37.06"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1025" min="9" style="0" width="11.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="15.07"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1025" min="10" style="0" width="11.52"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5066,15 +5070,25 @@
       <c r="B2" s="0" t="s">
         <v>212</v>
       </c>
-      <c r="E2" s="3"/>
+      <c r="C2" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="D2" s="0" t="n">
+        <v>18002437888</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>213</v>
+      </c>
       <c r="F2" s="5" t="s">
         <v>69</v>
       </c>
       <c r="G2" s="4"/>
-      <c r="H2" s="4"/>
+      <c r="H2" s="0" t="n">
+        <v>250</v>
+      </c>
     </row>
   </sheetData>
-  <dataValidations count="3">
+  <dataValidations count="2">
     <dataValidation allowBlank="false" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="F2" type="list">
       <formula1>Boolean</formula1>
       <formula2>0</formula2>
@@ -5083,11 +5097,10 @@
       <formula1>0</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="H2" type="decimal">
-      <formula1>0</formula1>
-      <formula2>100</formula2>
-    </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="E2" r:id="rId1" display="http://eap.com"/>
+  </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="1" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -5157,10 +5170,10 @@
     </row>
     <row r="2" customFormat="false" ht="248.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C2" s="0" t="s">
         <v>18</v>
@@ -5169,14 +5182,14 @@
         <v>8009889789</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="F2" s="5" t="s">
         <v>69</v>
       </c>
       <c r="G2" s="4"/>
       <c r="I2" s="6" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
   </sheetData>
@@ -5269,10 +5282,10 @@
     </row>
     <row r="2" customFormat="false" ht="293.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="C2" s="0" t="s">
         <v>18</v>
@@ -5281,7 +5294,7 @@
         <v>8009889789</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="F2" s="5" t="s">
         <v>69</v>
@@ -5291,7 +5304,7 @@
       </c>
       <c r="H2" s="4"/>
       <c r="I2" s="6" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="J2" s="0" t="n">
         <v>8009889789</v>
@@ -5386,16 +5399,19 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>222</v>
+        <v>223</v>
+      </c>
+      <c r="C2" s="0" t="s">
+        <v>18</v>
       </c>
       <c r="D2" s="0" t="n">
         <v>8009889789</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="F2" s="5" t="s">
         <v>69</v>
@@ -5407,16 +5423,19 @@
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>225</v>
+        <v>226</v>
+      </c>
+      <c r="C3" s="0" t="s">
+        <v>18</v>
       </c>
       <c r="D3" s="0" t="n">
         <v>8082342344</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="F3" s="5"/>
       <c r="G3" s="4"/>
@@ -5505,10 +5524,10 @@
         <v>125</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="AMH1" s="0"/>
       <c r="AMI1" s="0"/>
@@ -5516,16 +5535,19 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>229</v>
+        <v>230</v>
+      </c>
+      <c r="C2" s="0" t="s">
+        <v>18</v>
       </c>
       <c r="D2" s="0" t="n">
         <v>8009889789</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="F2" s="5" t="s">
         <v>69</v>
@@ -5622,10 +5644,10 @@
         <v>125</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="L1" s="0"/>
       <c r="M1" s="0"/>
@@ -5633,16 +5655,19 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>229</v>
+        <v>230</v>
+      </c>
+      <c r="C2" s="0" t="s">
+        <v>18</v>
       </c>
       <c r="D2" s="0" t="n">
         <v>8009889789</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="F2" s="5" t="s">
         <v>69</v>
@@ -5722,10 +5747,10 @@
         <v>45</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>125</v>
@@ -5742,10 +5767,13 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>234</v>
+        <v>235</v>
+      </c>
+      <c r="C2" s="0" t="s">
+        <v>18</v>
       </c>
       <c r="D2" s="0" t="n">
         <v>8009889789</v>
@@ -5828,10 +5856,10 @@
         <v>45</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>125</v>
@@ -5851,10 +5879,13 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>236</v>
+        <v>237</v>
+      </c>
+      <c r="C2" s="0" t="s">
+        <v>18</v>
       </c>
       <c r="D2" s="0" t="n">
         <v>8009889789</v>
@@ -5922,40 +5953,40 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B1" s="0" t="s">
         <v>25</v>
       </c>
       <c r="C1" s="0" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="D1" s="0" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="E1" s="0" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="F1" s="0" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="G1" s="0" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="H1" s="0" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="I1" s="0" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="J1" s="0" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="K1" s="0" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="L1" s="0" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6054,7 +6085,7 @@
         <v>2903</v>
       </c>
       <c r="C8" s="0" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="K8" s="0" t="n">
         <v>100000</v>
@@ -6099,7 +6130,7 @@
         <v>2903</v>
       </c>
       <c r="C11" s="0" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="G11" s="5" t="n">
         <f aca="false">TRUE()</f>
@@ -6143,34 +6174,34 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="C1" s="0" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="D1" s="0" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="E1" s="0" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="F1" s="0" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="G1" s="0" t="s">
         <v>95</v>
       </c>
       <c r="H1" s="0" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="I1" s="0" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="J1" s="0" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6178,7 +6209,7 @@
         <v>69</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C2" s="0" t="s">
         <v>61</v>
@@ -6193,13 +6224,13 @@
         <v>117</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="H2" s="0" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="I2" s="0" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="J2" s="0" t="s">
         <v>144</v>
@@ -6210,7 +6241,7 @@
         <v>106</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="C3" s="0" t="s">
         <v>78</v>
@@ -6222,16 +6253,16 @@
         <v>63</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="H3" s="0" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="I3" s="0" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="J3" s="0" t="s">
         <v>139</v>
@@ -6239,49 +6270,49 @@
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="0" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="G4" s="0" t="s">
         <v>109</v>
       </c>
       <c r="H4" s="0" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="I4" s="0" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="0" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="G5" s="0" t="s">
         <v>102</v>
       </c>
       <c r="H5" s="0" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="0" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="H6" s="0" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="0" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="H7" s="0" t="s">
         <v>72</v>
@@ -6289,182 +6320,182 @@
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="0" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="0" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="0" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="0" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="0" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="0" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="0" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="0" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="0" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="0" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="0" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="0" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="0" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="0" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="0" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="0" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="0" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="0" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="0" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="0" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="0" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="0" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="0" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="0" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="0" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="0" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="0" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="0" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="0" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="0" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="0" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="0" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B40" s="0" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B41" s="0" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B42" s="0" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B43" s="0" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6474,37 +6505,37 @@
     </row>
     <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B45" s="0" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B46" s="0" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B47" s="0" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B48" s="0" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B49" s="0" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B50" s="0" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B51" s="0" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Data migration for HRA.  Change base for 401k. Add docs from Mutual of Omaha.
</commit_message>
<xml_diff>
--- a/docs/data_import_example.xlsx
+++ b/docs/data_import_example.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="34"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="27"/>
   </bookViews>
   <sheets>
     <sheet name="Locations" sheetId="1" state="visible" r:id="rId2"/>
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="935" uniqueCount="323">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="934" uniqueCount="323">
   <si>
     <t xml:space="preserve">code</t>
   </si>
@@ -751,7 +751,7 @@
     <t xml:space="preserve">AEAP332</t>
   </si>
   <si>
-    <t xml:space="preserve">employee assistance</t>
+    <t xml:space="preserve">Employee Assistance</t>
   </si>
   <si>
     <t xml:space="preserve">http://eap.com</t>
@@ -1163,7 +1163,7 @@
     <numFmt numFmtId="165" formatCode="MM/DD/YY"/>
     <numFmt numFmtId="166" formatCode="&quot;TRUE&quot;;&quot;TRUE&quot;;&quot;FALSE&quot;"/>
   </numFmts>
-  <fonts count="18">
+  <fonts count="17">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -1279,11 +1279,6 @@
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="9">
@@ -1433,7 +1428,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1464,10 +1459,6 @@
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -3550,7 +3541,7 @@
       <c r="H2" s="0" t="n">
         <v>100</v>
       </c>
-      <c r="I2" s="8" t="s">
+      <c r="I2" s="6" t="s">
         <v>163</v>
       </c>
       <c r="J2" s="0" t="n">
@@ -4006,7 +3997,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="6.73"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="0" width="37.06"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="16.48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="20.55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="20.56"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1025" min="11" style="0" width="11.52"/>
   </cols>
   <sheetData>
@@ -4125,8 +4116,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="13.88"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="6.73"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="0" width="37.06"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="20.56"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="20.55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="9" style="0" width="20.56"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1025" min="11" style="0" width="11.52"/>
   </cols>
   <sheetData>
@@ -4247,9 +4237,8 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="6.73"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="0" width="37.06"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="20.56"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="20.55"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="11" style="0" width="37.06"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1025" min="13" style="0" width="11.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="10" style="0" width="37.06"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1025" min="12" style="0" width="11.52"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4280,11 +4269,9 @@
       <c r="I1" s="1" t="s">
         <v>203</v>
       </c>
-      <c r="J1" s="1" t="s">
-        <v>199</v>
-      </c>
+      <c r="J1" s="0"/>
       <c r="K1" s="0"/>
-      <c r="L1" s="0"/>
+      <c r="AMB1" s="0"/>
       <c r="AMC1" s="0"/>
       <c r="AMD1" s="0"/>
       <c r="AME1" s="0"/>
@@ -4318,9 +4305,6 @@
         <v>0</v>
       </c>
       <c r="I2" s="4"/>
-      <c r="J2" s="0" t="n">
-        <v>120</v>
-      </c>
     </row>
   </sheetData>
   <dataValidations count="4">
@@ -4370,7 +4354,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="0" width="37.06"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="9" style="0" width="40.88"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="27.45"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="20.55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="20.56"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1025" min="13" style="0" width="11.52"/>
   </cols>
   <sheetData>
@@ -5020,7 +5004,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="15.94"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="6.73"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="0" width="37.06"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="15.07"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="15.08"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1025" min="10" style="0" width="11.52"/>
   </cols>
   <sheetData>

</xml_diff>

<commit_message>
Fix standalond ADD plans.
</commit_message>
<xml_diff>
--- a/docs/data_import_example.xlsx
+++ b/docs/data_import_example.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="27"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="17"/>
   </bookViews>
   <sheets>
     <sheet name="Locations" sheetId="1" state="visible" r:id="rId2"/>
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="934" uniqueCount="323">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="936" uniqueCount="321">
   <si>
     <t xml:space="preserve">code</t>
   </si>
@@ -632,12 +632,6 @@
 65-69,41.15%
 70-74,67.04%
 75+,67.04%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">salary multiple death benefit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">salary multiple dismemberment benefit</t>
   </si>
   <si>
     <t xml:space="preserve">Accidental Death and Dismemberment</t>
@@ -1163,7 +1157,7 @@
     <numFmt numFmtId="165" formatCode="MM/DD/YY"/>
     <numFmt numFmtId="166" formatCode="&quot;TRUE&quot;;&quot;TRUE&quot;;&quot;FALSE&quot;"/>
   </numFmts>
-  <fonts count="17">
+  <fonts count="18">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -1279,6 +1273,11 @@
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="9">
@@ -1428,7 +1427,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1459,6 +1458,10 @@
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -2758,7 +2761,9 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="6.73"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="0" width="37.06"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="15.08"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="10" style="0" width="42.62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="25.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="20.63"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="21.1"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="35.23"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1025" min="14" style="0" width="11.52"/>
   </cols>
@@ -2792,16 +2797,13 @@
         <v>125</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>151</v>
+        <v>165</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>152</v>
+        <v>166</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>175</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>176</v>
+        <v>167</v>
       </c>
       <c r="ALX1" s="0"/>
       <c r="ALY1" s="0"/>
@@ -2822,7 +2824,7 @@
         <v>160</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="C2" s="4" t="s">
         <v>18</v>
@@ -2843,17 +2845,14 @@
       <c r="I2" s="6" t="s">
         <v>163</v>
       </c>
-      <c r="J2" s="6" t="n">
-        <v>25000</v>
-      </c>
-      <c r="K2" s="6" t="n">
-        <v>500000</v>
+      <c r="J2" s="0" t="n">
+        <v>20000</v>
+      </c>
+      <c r="K2" s="0" t="n">
+        <v>100000</v>
       </c>
       <c r="L2" s="0" t="n">
-        <v>2</v>
-      </c>
-      <c r="M2" s="0" t="n">
-        <v>2</v>
+        <v>200000</v>
       </c>
     </row>
   </sheetData>
@@ -3352,10 +3351,10 @@
         <v>125</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="L1" s="0"/>
       <c r="M1" s="0"/>
@@ -3363,10 +3362,10 @@
     </row>
     <row r="2" customFormat="false" ht="125.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="C2" s="4" t="s">
         <v>18</v>
@@ -3375,7 +3374,7 @@
         <v>8009889789</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="F2" s="5" t="s">
         <v>69</v>
@@ -3396,10 +3395,10 @@
     </row>
     <row r="3" customFormat="false" ht="125.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="C3" s="4" t="s">
         <v>18</v>
@@ -3408,7 +3407,7 @@
         <v>8009889789</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="F3" s="5" t="s">
         <v>69</v>
@@ -3511,19 +3510,19 @@
         <v>125</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="AMJ1" s="0"/>
     </row>
     <row r="2" customFormat="false" ht="125.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C2" s="4" t="s">
         <v>18</v>
@@ -3532,7 +3531,7 @@
         <v>8009889789</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="F2" s="5" t="s">
         <v>69</v>
@@ -3646,10 +3645,10 @@
         <v>125</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="L1" s="0"/>
       <c r="M1" s="0"/>
@@ -3664,10 +3663,10 @@
     </row>
     <row r="2" customFormat="false" ht="73.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="C2" s="4" t="s">
         <v>18</v>
@@ -3676,7 +3675,7 @@
         <v>8009889789</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="F2" s="5" t="s">
         <v>69</v>
@@ -3686,7 +3685,7 @@
         <v>0</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="J2" s="0" t="n">
         <v>60</v>
@@ -3779,10 +3778,10 @@
         <v>125</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="L1" s="0"/>
       <c r="M1" s="0"/>
@@ -3797,10 +3796,10 @@
     </row>
     <row r="2" customFormat="false" ht="73.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="C2" s="4" t="s">
         <v>18</v>
@@ -3809,7 +3808,7 @@
         <v>8009889789</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="F2" s="5" t="s">
         <v>69</v>
@@ -3819,7 +3818,7 @@
         <v>100</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="J2" s="0" t="n">
         <v>60</v>
@@ -3909,7 +3908,7 @@
         <v>125</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="K1" s="0"/>
       <c r="L1" s="0"/>
@@ -3924,10 +3923,10 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C2" s="4" t="s">
         <v>18</v>
@@ -3936,7 +3935,7 @@
         <v>8009889789</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="F2" s="5" t="s">
         <v>69</v>
@@ -4030,7 +4029,7 @@
         <v>125</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="AMA1" s="0"/>
       <c r="AMB1" s="0"/>
@@ -4045,10 +4044,10 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C2" s="4" t="s">
         <v>18</v>
@@ -4057,7 +4056,7 @@
         <v>8009889789</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="F2" s="5" t="s">
         <v>69</v>
@@ -4149,7 +4148,7 @@
         <v>125</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="ALZ1" s="0"/>
       <c r="AMA1" s="0"/>
@@ -4165,10 +4164,10 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="C2" s="4" t="s">
         <v>18</v>
@@ -4177,7 +4176,7 @@
         <v>8009889789</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="F2" s="5" t="s">
         <v>69</v>
@@ -4267,7 +4266,7 @@
         <v>124</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="J1" s="0"/>
       <c r="K1" s="0"/>
@@ -4283,10 +4282,10 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="C2" s="4" t="s">
         <v>18</v>
@@ -4295,7 +4294,7 @@
         <v>8009889789</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="F2" s="5" t="s">
         <v>69</v>
@@ -4387,13 +4386,13 @@
         <v>125</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="AME1" s="0"/>
       <c r="AMF1" s="0"/>
@@ -4404,10 +4403,10 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="C2" s="0" t="s">
         <v>18</v>
@@ -4416,7 +4415,7 @@
         <v>8009889789</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F2" s="5" t="s">
         <v>69</v>
@@ -5049,10 +5048,10 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="C2" s="0" t="s">
         <v>18</v>
@@ -5061,7 +5060,7 @@
         <v>18002437888</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="F2" s="5" t="s">
         <v>69</v>
@@ -5154,10 +5153,10 @@
     </row>
     <row r="2" customFormat="false" ht="248.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="C2" s="0" t="s">
         <v>18</v>
@@ -5166,14 +5165,14 @@
         <v>8009889789</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="F2" s="5" t="s">
         <v>69</v>
       </c>
       <c r="G2" s="4"/>
       <c r="I2" s="6" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
     </row>
   </sheetData>
@@ -5266,10 +5265,10 @@
     </row>
     <row r="2" customFormat="false" ht="293.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="C2" s="0" t="s">
         <v>18</v>
@@ -5278,7 +5277,7 @@
         <v>8009889789</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="F2" s="5" t="s">
         <v>69</v>
@@ -5288,13 +5287,13 @@
       </c>
       <c r="H2" s="4"/>
       <c r="I2" s="6" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="J2" s="0" t="n">
         <v>8009889789</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
   </sheetData>
@@ -5381,12 +5380,12 @@
       <c r="AMI1" s="0"/>
       <c r="AMJ1" s="0"/>
     </row>
-    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="42.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="C2" s="0" t="s">
         <v>18</v>
@@ -5395,7 +5394,7 @@
         <v>8009889789</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="F2" s="5" t="s">
         <v>69</v>
@@ -5404,13 +5403,16 @@
       <c r="H2" s="4" t="n">
         <v>0.8</v>
       </c>
-    </row>
-    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I2" s="8" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="42.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="C3" s="0" t="s">
         <v>18</v>
@@ -5419,12 +5421,15 @@
         <v>8082342344</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="F3" s="5"/>
       <c r="G3" s="4"/>
       <c r="H3" s="4" t="n">
         <v>0.5</v>
+      </c>
+      <c r="I3" s="8" t="s">
+        <v>137</v>
       </c>
     </row>
   </sheetData>
@@ -5508,21 +5513,21 @@
         <v>125</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="AMH1" s="0"/>
       <c r="AMI1" s="0"/>
       <c r="AMJ1" s="0"/>
     </row>
-    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="42.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="C2" s="0" t="s">
         <v>18</v>
@@ -5531,7 +5536,7 @@
         <v>8009889789</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="F2" s="5" t="s">
         <v>69</v>
@@ -5540,6 +5545,9 @@
       <c r="H2" s="4" t="n">
         <v>0.8</v>
       </c>
+      <c r="I2" s="8" t="s">
+        <v>137</v>
+      </c>
       <c r="J2" s="0" t="n">
         <v>150000</v>
       </c>
@@ -5549,10 +5557,6 @@
     </row>
   </sheetData>
   <dataValidations count="3">
-    <dataValidation allowBlank="false" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="F2" type="list">
-      <formula1>Boolean</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
     <dataValidation allowBlank="false" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="G2" type="decimal">
       <formula1>0</formula1>
       <formula2>0</formula2>
@@ -5560,6 +5564,10 @@
     <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="H2" type="decimal">
       <formula1>0</formula1>
       <formula2>100</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="F2" type="list">
+      <formula1>Boolean</formula1>
+      <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -5628,10 +5636,10 @@
         <v>125</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="L1" s="0"/>
       <c r="M1" s="0"/>
@@ -5639,10 +5647,10 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="C2" s="0" t="s">
         <v>18</v>
@@ -5651,7 +5659,7 @@
         <v>8009889789</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="F2" s="5" t="s">
         <v>69</v>
@@ -5731,10 +5739,10 @@
         <v>45</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>125</v>
@@ -5751,10 +5759,10 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="C2" s="0" t="s">
         <v>18</v>
@@ -5763,7 +5771,7 @@
         <v>8009889789</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="F2" s="5" t="s">
         <v>69</v>
@@ -5840,10 +5848,10 @@
         <v>45</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>125</v>
@@ -5863,10 +5871,10 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="C2" s="0" t="s">
         <v>18</v>
@@ -5875,7 +5883,7 @@
         <v>8009889789</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="F2" s="5" t="s">
         <v>69</v>
@@ -5937,40 +5945,40 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="B1" s="0" t="s">
         <v>25</v>
       </c>
       <c r="C1" s="0" t="s">
+        <v>237</v>
+      </c>
+      <c r="D1" s="0" t="s">
+        <v>238</v>
+      </c>
+      <c r="E1" s="0" t="s">
         <v>239</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="F1" s="0" t="s">
         <v>240</v>
       </c>
-      <c r="E1" s="0" t="s">
+      <c r="G1" s="0" t="s">
         <v>241</v>
       </c>
-      <c r="F1" s="0" t="s">
+      <c r="H1" s="0" t="s">
         <v>242</v>
       </c>
-      <c r="G1" s="0" t="s">
+      <c r="I1" s="0" t="s">
         <v>243</v>
       </c>
-      <c r="H1" s="0" t="s">
+      <c r="J1" s="0" t="s">
         <v>244</v>
       </c>
-      <c r="I1" s="0" t="s">
+      <c r="K1" s="0" t="s">
         <v>245</v>
       </c>
-      <c r="J1" s="0" t="s">
+      <c r="L1" s="0" t="s">
         <v>246</v>
-      </c>
-      <c r="K1" s="0" t="s">
-        <v>247</v>
-      </c>
-      <c r="L1" s="0" t="s">
-        <v>248</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6027,7 +6035,7 @@
         <v>2903</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="K5" s="0" t="n">
         <v>10000</v>
@@ -6041,7 +6049,7 @@
         <v>2903</v>
       </c>
       <c r="C6" s="0" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="K6" s="0" t="n">
         <v>20000</v>
@@ -6069,7 +6077,7 @@
         <v>2903</v>
       </c>
       <c r="C8" s="0" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="K8" s="0" t="n">
         <v>100000</v>
@@ -6086,7 +6094,7 @@
         <v>2903</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="K9" s="0" t="n">
         <v>1500</v>
@@ -6100,7 +6108,7 @@
         <v>2903</v>
       </c>
       <c r="C10" s="0" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="K10" s="0" t="n">
         <v>10000</v>
@@ -6114,7 +6122,7 @@
         <v>2903</v>
       </c>
       <c r="C11" s="0" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="G11" s="5" t="n">
         <f aca="false">TRUE()</f>
@@ -6158,34 +6166,34 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
+        <v>249</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>250</v>
+      </c>
+      <c r="C1" s="0" t="s">
         <v>251</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="D1" s="0" t="s">
         <v>252</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="E1" s="0" t="s">
         <v>253</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="F1" s="0" t="s">
         <v>254</v>
-      </c>
-      <c r="E1" s="0" t="s">
-        <v>255</v>
-      </c>
-      <c r="F1" s="0" t="s">
-        <v>256</v>
       </c>
       <c r="G1" s="0" t="s">
         <v>95</v>
       </c>
       <c r="H1" s="0" t="s">
+        <v>255</v>
+      </c>
+      <c r="I1" s="0" t="s">
+        <v>256</v>
+      </c>
+      <c r="J1" s="0" t="s">
         <v>257</v>
-      </c>
-      <c r="I1" s="0" t="s">
-        <v>258</v>
-      </c>
-      <c r="J1" s="0" t="s">
-        <v>259</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6193,7 +6201,7 @@
         <v>69</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="C2" s="0" t="s">
         <v>61</v>
@@ -6208,13 +6216,13 @@
         <v>117</v>
       </c>
       <c r="G2" s="0" t="s">
+        <v>259</v>
+      </c>
+      <c r="H2" s="0" t="s">
+        <v>260</v>
+      </c>
+      <c r="I2" s="0" t="s">
         <v>261</v>
-      </c>
-      <c r="H2" s="0" t="s">
-        <v>262</v>
-      </c>
-      <c r="I2" s="0" t="s">
-        <v>263</v>
       </c>
       <c r="J2" s="0" t="s">
         <v>144</v>
@@ -6225,7 +6233,7 @@
         <v>106</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="C3" s="0" t="s">
         <v>78</v>
@@ -6237,16 +6245,16 @@
         <v>63</v>
       </c>
       <c r="F3" s="0" t="s">
+        <v>263</v>
+      </c>
+      <c r="G3" s="0" t="s">
+        <v>264</v>
+      </c>
+      <c r="H3" s="0" t="s">
         <v>265</v>
       </c>
-      <c r="G3" s="0" t="s">
+      <c r="I3" s="0" t="s">
         <v>266</v>
-      </c>
-      <c r="H3" s="0" t="s">
-        <v>267</v>
-      </c>
-      <c r="I3" s="0" t="s">
-        <v>268</v>
       </c>
       <c r="J3" s="0" t="s">
         <v>139</v>
@@ -6254,49 +6262,49 @@
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="0" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="G4" s="0" t="s">
         <v>109</v>
       </c>
       <c r="H4" s="0" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="I4" s="0" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="0" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="G5" s="0" t="s">
         <v>102</v>
       </c>
       <c r="H5" s="0" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="0" t="s">
+        <v>274</v>
+      </c>
+      <c r="G6" s="0" t="s">
+        <v>275</v>
+      </c>
+      <c r="H6" s="0" t="s">
         <v>276</v>
-      </c>
-      <c r="G6" s="0" t="s">
-        <v>277</v>
-      </c>
-      <c r="H6" s="0" t="s">
-        <v>278</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="0" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="H7" s="0" t="s">
         <v>72</v>
@@ -6304,182 +6312,182 @@
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="0" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="0" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="0" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="0" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="0" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="0" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="0" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="0" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="0" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="0" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="0" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="0" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="0" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="0" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="0" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="0" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="0" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="0" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="0" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="0" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="0" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="0" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="0" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="0" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="0" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="0" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="0" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="0" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="0" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="0" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="0" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="0" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B40" s="0" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B41" s="0" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B42" s="0" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B43" s="0" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6489,37 +6497,37 @@
     </row>
     <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B45" s="0" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B46" s="0" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B47" s="0" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B48" s="0" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B49" s="0" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B50" s="0" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B51" s="0" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
     </row>
   </sheetData>
@@ -7210,7 +7218,7 @@
       <c r="AMI1" s="0"/>
       <c r="AMJ1" s="0"/>
     </row>
-    <row r="2" s="4" customFormat="true" ht="40.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" s="4" customFormat="true" ht="42.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
         <v>134</v>
       </c>

</xml_diff>

<commit_message>
Add support to importer for premium_matrix that has one and only one set premium. Fix HospitalConfinementPlan (add TieredElectionMixin)
</commit_message>
<xml_diff>
--- a/docs/data_import_example.xlsx
+++ b/docs/data_import_example.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="17"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="35"/>
   </bookViews>
   <sheets>
     <sheet name="Locations" sheetId="1" state="visible" r:id="rId2"/>
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="936" uniqueCount="321">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="937" uniqueCount="321">
   <si>
     <t xml:space="preserve">code</t>
   </si>
@@ -1152,10 +1152,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="MM/DD/YY"/>
     <numFmt numFmtId="166" formatCode="&quot;TRUE&quot;;&quot;TRUE&quot;;&quot;FALSE&quot;"/>
+    <numFmt numFmtId="167" formatCode="[$$-409]#,##0.00;[RED]\-[$$-409]#,##0.00"/>
   </numFmts>
   <fonts count="18">
     <font>
@@ -1427,7 +1428,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1462,6 +1463,10 @@
     </xf>
     <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -4070,10 +4075,6 @@
     </row>
   </sheetData>
   <dataValidations count="4">
-    <dataValidation allowBlank="false" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="F2 I2" type="list">
-      <formula1>Boolean</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
     <dataValidation allowBlank="false" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="G2" type="decimal">
       <formula1>0</formula1>
       <formula2>0</formula2>
@@ -4081,6 +4082,10 @@
     <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="H2" type="decimal">
       <formula1>0</formula1>
       <formula2>100</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="F2 I2" type="list">
+      <formula1>Boolean</formula1>
+      <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="false" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="C2" type="list">
       <formula1>Carriers</formula1>
@@ -5177,12 +5182,12 @@
     </row>
   </sheetData>
   <dataValidations count="2">
+    <dataValidation allowBlank="false" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="G2" type="decimal">
+      <formula1>0</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
     <dataValidation allowBlank="false" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="F2" type="list">
       <formula1>Boolean</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="false" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="G2" type="decimal">
-      <formula1>0</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -5298,10 +5303,6 @@
     </row>
   </sheetData>
   <dataValidations count="3">
-    <dataValidation allowBlank="false" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="F2" type="list">
-      <formula1>Boolean</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
     <dataValidation allowBlank="false" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="G2" type="decimal">
       <formula1>0</formula1>
       <formula2>0</formula2>
@@ -5309,6 +5310,10 @@
     <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="H2" type="decimal">
       <formula1>0</formula1>
       <formula2>100</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="F2" type="list">
+      <formula1>Boolean</formula1>
+      <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
@@ -5403,7 +5408,7 @@
       <c r="H2" s="4" t="n">
         <v>0.8</v>
       </c>
-      <c r="I2" s="8" t="s">
+      <c r="I2" s="6" t="s">
         <v>137</v>
       </c>
     </row>
@@ -5428,16 +5433,12 @@
       <c r="H3" s="4" t="n">
         <v>0.5</v>
       </c>
-      <c r="I3" s="8" t="s">
+      <c r="I3" s="6" t="s">
         <v>137</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="3">
-    <dataValidation allowBlank="false" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="F2:F3" type="list">
-      <formula1>Boolean</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
     <dataValidation allowBlank="false" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="G2:G3" type="decimal">
       <formula1>0</formula1>
       <formula2>0</formula2>
@@ -5445,6 +5446,10 @@
     <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="H2:H3" type="decimal">
       <formula1>0</formula1>
       <formula2>100</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="F2:F3" type="list">
+      <formula1>Boolean</formula1>
+      <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
@@ -5545,7 +5550,7 @@
       <c r="H2" s="4" t="n">
         <v>0.8</v>
       </c>
-      <c r="I2" s="8" t="s">
+      <c r="I2" s="6" t="s">
         <v>137</v>
       </c>
       <c r="J2" s="0" t="n">
@@ -5645,7 +5650,7 @@
       <c r="M1" s="0"/>
       <c r="N1" s="0"/>
     </row>
-    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="42.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
         <v>227</v>
       </c>
@@ -5667,6 +5672,9 @@
       <c r="G2" s="4"/>
       <c r="H2" s="4" t="n">
         <v>0.8</v>
+      </c>
+      <c r="I2" s="8" t="s">
+        <v>137</v>
       </c>
       <c r="J2" s="0" t="n">
         <v>150000</v>
@@ -5778,6 +5786,9 @@
       </c>
       <c r="G2" s="0" t="n">
         <v>200</v>
+      </c>
+      <c r="I2" s="9" t="n">
+        <v>250</v>
       </c>
     </row>
   </sheetData>
@@ -5891,16 +5902,15 @@
       <c r="G2" s="0" t="n">
         <v>200</v>
       </c>
+      <c r="I2" s="9" t="n">
+        <v>200</v>
+      </c>
       <c r="J2" s="0" t="n">
         <v>2000</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="3">
-    <dataValidation allowBlank="false" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="F2" type="list">
-      <formula1>Boolean</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
     <dataValidation allowBlank="false" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="G2" type="decimal">
       <formula1>0</formula1>
       <formula2>0</formula2>
@@ -5908,6 +5918,10 @@
     <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="H2" type="decimal">
       <formula1>0</formula1>
       <formula2>100</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="F2" type="list">
+      <formula1>Boolean</formula1>
+      <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
   <hyperlinks>

</xml_diff>

<commit_message>
Display FSA Medical and FSA Dependent under the same header. Fix prefix for identity theft. Add premium_matrix as a text field to plan so it can be entered/displayed in admin forms. Fix admin templates for Core benefits.
</commit_message>
<xml_diff>
--- a/docs/data_import_example.xlsx
+++ b/docs/data_import_example.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="35"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="36"/>
   </bookViews>
   <sheets>
     <sheet name="Locations" sheetId="1" state="visible" r:id="rId2"/>
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="937" uniqueCount="321">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="938" uniqueCount="323">
   <si>
     <t xml:space="preserve">code</t>
   </si>
@@ -707,6 +707,9 @@
   </si>
   <si>
     <t xml:space="preserve">minimum contribution</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dependent Flexible Spending Account</t>
   </si>
   <si>
     <t xml:space="preserve">HSA82289</t>
@@ -891,6 +894,9 @@
   </si>
   <si>
     <t xml:space="preserve">Identity Theft</t>
+  </si>
+  <si>
+    <t xml:space="preserve">employee_only,$250</t>
   </si>
   <si>
     <t xml:space="preserve">enrollment year</t>
@@ -1428,7 +1434,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1466,6 +1472,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -4052,7 +4062,7 @@
         <v>194</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="C2" s="4" t="s">
         <v>18</v>
@@ -4169,10 +4179,10 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="C2" s="4" t="s">
         <v>18</v>
@@ -4181,7 +4191,7 @@
         <v>8009889789</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="F2" s="5" t="s">
         <v>69</v>
@@ -4271,7 +4281,7 @@
         <v>124</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="J1" s="0"/>
       <c r="K1" s="0"/>
@@ -4287,10 +4297,10 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="C2" s="4" t="s">
         <v>18</v>
@@ -4299,7 +4309,7 @@
         <v>8009889789</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="F2" s="5" t="s">
         <v>69</v>
@@ -4391,10 +4401,10 @@
         <v>125</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="L1" s="1" t="s">
         <v>197</v>
@@ -4408,10 +4418,10 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="C2" s="0" t="s">
         <v>18</v>
@@ -4420,7 +4430,7 @@
         <v>8009889789</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="F2" s="5" t="s">
         <v>69</v>
@@ -5053,10 +5063,10 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="C2" s="0" t="s">
         <v>18</v>
@@ -5065,7 +5075,7 @@
         <v>18002437888</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="F2" s="5" t="s">
         <v>69</v>
@@ -5158,10 +5168,10 @@
     </row>
     <row r="2" customFormat="false" ht="248.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C2" s="0" t="s">
         <v>18</v>
@@ -5170,14 +5180,14 @@
         <v>8009889789</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="F2" s="5" t="s">
         <v>69</v>
       </c>
       <c r="G2" s="4"/>
       <c r="I2" s="6" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
     </row>
   </sheetData>
@@ -5270,10 +5280,10 @@
     </row>
     <row r="2" customFormat="false" ht="293.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="C2" s="0" t="s">
         <v>18</v>
@@ -5282,7 +5292,7 @@
         <v>8009889789</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="F2" s="5" t="s">
         <v>69</v>
@@ -5292,13 +5302,13 @@
       </c>
       <c r="H2" s="4"/>
       <c r="I2" s="6" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="J2" s="0" t="n">
         <v>8009889789</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
   </sheetData>
@@ -5387,10 +5397,10 @@
     </row>
     <row r="2" customFormat="false" ht="42.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="C2" s="0" t="s">
         <v>18</v>
@@ -5399,7 +5409,7 @@
         <v>8009889789</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="F2" s="5" t="s">
         <v>69</v>
@@ -5414,10 +5424,10 @@
     </row>
     <row r="3" customFormat="false" ht="42.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="C3" s="0" t="s">
         <v>18</v>
@@ -5426,7 +5436,7 @@
         <v>8082342344</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="F3" s="5"/>
       <c r="G3" s="4"/>
@@ -5518,10 +5528,10 @@
         <v>125</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="AMH1" s="0"/>
       <c r="AMI1" s="0"/>
@@ -5529,10 +5539,10 @@
     </row>
     <row r="2" customFormat="false" ht="42.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C2" s="0" t="s">
         <v>18</v>
@@ -5541,7 +5551,7 @@
         <v>8009889789</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="F2" s="5" t="s">
         <v>69</v>
@@ -5641,10 +5651,10 @@
         <v>125</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="L1" s="0"/>
       <c r="M1" s="0"/>
@@ -5652,10 +5662,10 @@
     </row>
     <row r="2" customFormat="false" ht="42.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C2" s="0" t="s">
         <v>18</v>
@@ -5664,7 +5674,7 @@
         <v>8009889789</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="F2" s="5" t="s">
         <v>69</v>
@@ -5747,10 +5757,10 @@
         <v>45</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>125</v>
@@ -5767,10 +5777,10 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="C2" s="0" t="s">
         <v>18</v>
@@ -5779,7 +5789,7 @@
         <v>8009889789</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="F2" s="5" t="s">
         <v>69</v>
@@ -5859,10 +5869,10 @@
         <v>45</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>125</v>
@@ -5882,10 +5892,10 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="C2" s="0" t="s">
         <v>18</v>
@@ -5894,7 +5904,7 @@
         <v>8009889789</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="F2" s="5" t="s">
         <v>69</v>
@@ -5902,8 +5912,8 @@
       <c r="G2" s="0" t="n">
         <v>200</v>
       </c>
-      <c r="I2" s="9" t="n">
-        <v>200</v>
+      <c r="I2" s="10" t="s">
+        <v>237</v>
       </c>
       <c r="J2" s="0" t="n">
         <v>2000</v>
@@ -5959,40 +5969,40 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="B1" s="0" t="s">
         <v>25</v>
       </c>
       <c r="C1" s="0" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="D1" s="0" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="E1" s="0" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="F1" s="0" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="G1" s="0" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="H1" s="0" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="I1" s="0" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="J1" s="0" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="K1" s="0" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="L1" s="0" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6049,7 +6059,7 @@
         <v>2903</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="K5" s="0" t="n">
         <v>10000</v>
@@ -6091,7 +6101,7 @@
         <v>2903</v>
       </c>
       <c r="C8" s="0" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="K8" s="0" t="n">
         <v>100000</v>
@@ -6122,7 +6132,7 @@
         <v>2903</v>
       </c>
       <c r="C10" s="0" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="K10" s="0" t="n">
         <v>10000</v>
@@ -6136,7 +6146,7 @@
         <v>2903</v>
       </c>
       <c r="C11" s="0" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="G11" s="5" t="n">
         <f aca="false">TRUE()</f>
@@ -6180,34 +6190,34 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="C1" s="0" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="D1" s="0" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="E1" s="0" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="F1" s="0" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="G1" s="0" t="s">
         <v>95</v>
       </c>
       <c r="H1" s="0" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="I1" s="0" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="J1" s="0" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6215,7 +6225,7 @@
         <v>69</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="C2" s="0" t="s">
         <v>61</v>
@@ -6230,13 +6240,13 @@
         <v>117</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="H2" s="0" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="I2" s="0" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="J2" s="0" t="s">
         <v>144</v>
@@ -6247,7 +6257,7 @@
         <v>106</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="C3" s="0" t="s">
         <v>78</v>
@@ -6259,16 +6269,16 @@
         <v>63</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="H3" s="0" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="I3" s="0" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="J3" s="0" t="s">
         <v>139</v>
@@ -6276,49 +6286,49 @@
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="0" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="G4" s="0" t="s">
         <v>109</v>
       </c>
       <c r="H4" s="0" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="I4" s="0" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="0" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="G5" s="0" t="s">
         <v>102</v>
       </c>
       <c r="H5" s="0" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="0" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="H6" s="0" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="0" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="H7" s="0" t="s">
         <v>72</v>
@@ -6326,182 +6336,182 @@
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="0" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="0" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="0" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="0" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="0" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="0" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="0" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="0" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="0" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="0" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="0" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="0" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="0" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="0" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="0" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="0" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="0" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="0" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="0" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="0" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="0" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="0" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="0" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="0" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="0" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="0" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="0" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="0" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="0" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="0" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="0" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="0" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B40" s="0" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B41" s="0" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B42" s="0" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B43" s="0" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6511,37 +6521,37 @@
     </row>
     <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B45" s="0" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B46" s="0" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B47" s="0" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B48" s="0" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B49" s="0" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B50" s="0" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B51" s="0" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Lots of fixes for field validation, and test fixes.
</commit_message>
<xml_diff>
--- a/docs/data_import_example.xlsx
+++ b/docs/data_import_example.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="18"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="14"/>
   </bookViews>
   <sheets>
     <sheet name="Locations" sheetId="1" state="visible" r:id="rId2"/>
@@ -1429,7 +1429,7 @@
     <numFmt numFmtId="166" formatCode="&quot;TRUE&quot;;&quot;TRUE&quot;;&quot;FALSE&quot;"/>
     <numFmt numFmtId="167" formatCode="[$$-409]#,##0.00;[RED]\-[$$-409]#,##0.00"/>
   </numFmts>
-  <fonts count="18">
+  <fonts count="17">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -1545,11 +1545,6 @@
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="9">
@@ -1699,7 +1694,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1730,10 +1725,6 @@
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
@@ -3181,7 +3172,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="18.08"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="6.73"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="37.06"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="12.62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="12.63"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="45.25"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="16.48"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="16.97"/>
@@ -3277,7 +3268,7 @@
       <c r="H2" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="I2" s="8" t="s">
+      <c r="I2" s="6" t="s">
         <v>176</v>
       </c>
       <c r="J2" s="0" t="n">
@@ -4724,13 +4715,13 @@
       <formula1>0</formula1>
       <formula2>100</formula2>
     </dataValidation>
+    <dataValidation allowBlank="false" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="F2 I2" type="list">
+      <formula1>Boolean</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
     <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="J2" type="decimal">
       <formula1>0</formula1>
       <formula2>100</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="false" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="F2 I2" type="list">
-      <formula1>Boolean</formula1>
-      <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
@@ -6063,7 +6054,7 @@
       <c r="G2" s="0" t="n">
         <v>200</v>
       </c>
-      <c r="I2" s="9" t="n">
+      <c r="I2" s="8" t="n">
         <v>250</v>
       </c>
     </row>
@@ -6178,7 +6169,7 @@
       <c r="G2" s="0" t="n">
         <v>200</v>
       </c>
-      <c r="I2" s="10" t="s">
+      <c r="I2" s="9" t="s">
         <v>238</v>
       </c>
       <c r="J2" s="0" t="n">

</xml_diff>

<commit_message>
Fixes for stable before moving to wizard approach.
</commit_message>
<xml_diff>
--- a/docs/data_import_example.xlsx
+++ b/docs/data_import_example.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="14"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="8"/>
   </bookViews>
   <sheets>
     <sheet name="Locations" sheetId="1" state="visible" r:id="rId2"/>
@@ -3128,14 +3128,6 @@
     </row>
   </sheetData>
   <dataValidations count="4">
-    <dataValidation allowBlank="false" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="F2" type="list">
-      <formula1>Boolean</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="false" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="C2" type="list">
-      <formula1>Carriers</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
     <dataValidation allowBlank="false" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="G2" type="decimal">
       <formula1>0</formula1>
       <formula2>0</formula2>
@@ -3143,6 +3135,14 @@
     <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="H2" type="decimal">
       <formula1>0</formula1>
       <formula2>100</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="F2" type="list">
+      <formula1>Boolean</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="C2" type="list">
+      <formula1>Carriers</formula1>
+      <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
   <hyperlinks>

</xml_diff>